<commit_message>
Add PT1 start register fields
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_plan.xlsx
+++ b/tests/fixtures/sample_plan.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,11 +497,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>pt1_p_start_register</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>pt1_q_ms</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" t="n">
         <v>250</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>pt1_q_start_register</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalize demo-ready Modbus manager
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_plan.xlsx
+++ b/tests/fixtures/sample_plan.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,6 +522,60 @@
       </c>
       <c r="B10" t="n">
         <v>1300</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>remote_enabled</t>
+        </is>
+      </c>
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>remote_auto_control</t>
+        </is>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>remote_host</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>192.168.0.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>remote_port</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5025</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>remote_filename</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Bachmann_SPPC_EN_20260325_112003_001.dmd</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>